<commit_message>
Refresh authentic Stata 2.5.1 goldens and reconcile demo parity
</commit_message>
<xml_diff>
--- a/tests/testthat/golden/K01.xlsx
+++ b/tests/testthat/golden/K01.xlsx
@@ -114,7 +114,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -124,17 +124,13 @@
       <name val="Arial"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <b/>
       <name val="Arial"/>
     </font>
     <font>
@@ -146,6 +142,15 @@
       <sz val="10"/>
       <b/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
     </font>
     <font>
       <sz val="8"/>
@@ -165,7 +170,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -174,6 +179,62 @@
       <diagonal/>
     </border>
     <border/>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -184,8 +245,8 @@
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="thin"/>
-      <bottom style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -198,8 +259,8 @@
     <border>
       <left style="none"/>
       <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
       <diagonal style="none"/>
     </border>
   </borders>
@@ -209,111 +270,100 @@
   <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -336,72 +386,72 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="8" t="s">
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="12" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="12" t="s">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="14" t="s">
+      <c r="A5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -424,58 +474,58 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="8" t="s">
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="12" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="12" t="s">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="14" t="s">
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="8" t="s">
         <v>20</v>
       </c>
     </row>
@@ -511,26 +561,26 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="15" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="15" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="15" t="s">
         <v>26</v>
       </c>
     </row>
@@ -543,10 +593,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="15" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>